<commit_message>
Nouvelle palette (gris, orange, blanc cassé/beige) et rapport sans code
- Classeur Excel : en-têtes beige, entrées grises, résultats orange,
  courbes orange/gris
- Rapport Rmd/PDF : format rapport (aucun code visible), réponses
  encadrées, mêmes résultats

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JKxMnLxAqKW9FU7zDuTH4e
</commit_message>
<xml_diff>
--- a/Projet_ENSAE_Finance_de_Marche.xlsx
+++ b/Projet_ENSAE_Finance_de_Marche.xlsx
@@ -38,17 +38,17 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="001A1A1A"/>
+      <color rgb="003B3B3B"/>
       <sz val="14"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="001A1A1A"/>
+      <color rgb="003B3B3B"/>
       <sz val="11"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="0038761D"/>
+      <color rgb="00C55A11"/>
       <sz val="11"/>
     </font>
   </fonts>
@@ -61,12 +61,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFFCC"/>
+        <fgColor rgb="00F1E8D8"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00CCFFCC"/>
+        <fgColor rgb="00E7E5E0"/>
       </patternFill>
     </fill>
   </fills>
@@ -288,7 +288,7 @@
           <spPr>
             <a:ln w="25000">
               <a:solidFill>
-                <a:srgbClr val="38761D"/>
+                <a:srgbClr val="C55A11"/>
               </a:solidFill>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -409,7 +409,7 @@
           <spPr>
             <a:ln w="25000">
               <a:solidFill>
-                <a:srgbClr val="38761D"/>
+                <a:srgbClr val="C55A11"/>
               </a:solidFill>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -444,7 +444,7 @@
             <a:ln w="25000">
               <a:noFill/>
               <a:solidFill>
-                <a:srgbClr val="B8860B"/>
+                <a:srgbClr val="595959"/>
               </a:solidFill>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -915,7 +915,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Les cellules vertes contiennent les données d'entrée ; les résultats calculés sont en gras vert foncé.</t>
+          <t>Les cellules grises contiennent les données d'entrée ; les résultats calculés sont en gras orange.</t>
         </is>
       </c>
     </row>
@@ -970,7 +970,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Palette de couleurs autorisée (celle du Rmd) : jaune pâle #FFFFCC, vert pâle #CCFFCC et leurs déclinaisons foncées.</t>
+          <t>Palette de couleurs : gris, orange, blanc cassé / beige.</t>
         </is>
       </c>
     </row>

</xml_diff>